<commit_message>
Lanzar Beta-1.0.3 con nuevas skills y sincronizacion de catalogo.
Incluye nuevas clases de habilidad (stun/life_steal/dot), estados visuales en combate, sincronizacion automática de skills/imagenes desde Excel y actualizacion de recursos/versionado.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/eventos.xlsx
+++ b/public/resources/eventos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8724AE-15B3-4C23-9A3B-120BC8FE203D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8E5016-F203-4555-8465-00CDEE3CAD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
   <si>
     <t>nombre</t>
   </si>
@@ -166,6 +166,9 @@
   </si>
   <si>
     <t>Parallax</t>
+  </si>
+  <si>
+    <t>Darkseid</t>
   </si>
 </sst>
 </file>
@@ -652,7 +655,7 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="4" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="K3" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Actualiza cartas.xlsx y eventos.xlsx
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/eventos.xlsx
+++ b/public/resources/eventos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0645909-2867-447D-857D-1B48604EB6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CEA91B-2D3D-492F-95EA-EEFD6EA73E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -564,9 +564,6 @@
     <t>Los mayores genios y conquistadores del universo unen fuerzas en un combate que decidirá el destino de la humanidad.</t>
   </si>
   <si>
-    <t>Pyscho-Pirate</t>
-  </si>
-  <si>
     <t>Telos</t>
   </si>
   <si>
@@ -594,9 +591,6 @@
     <t>Reign</t>
   </si>
   <si>
-    <t>Superboy-Prime</t>
-  </si>
-  <si>
     <t>Ultraman</t>
   </si>
   <si>
@@ -739,6 +733,12 @@
   </si>
   <si>
     <t>Dex Starr</t>
+  </si>
+  <si>
+    <t>Superboy Prime</t>
+  </si>
+  <si>
+    <t>Psycho-Pirate</t>
   </si>
 </sst>
 </file>
@@ -1176,29 +1176,29 @@
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="E2" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>227</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>229</v>
       </c>
       <c r="I2" s="6"/>
       <c r="J2" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K2" s="6">
         <v>1</v>
@@ -1508,7 +1508,7 @@
         <v>138</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>140</v>
@@ -1670,7 +1670,7 @@
         <v>155</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>24</v>
@@ -1694,31 +1694,31 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="E15" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="J15" s="6" t="s">
         <v>233</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>235</v>
       </c>
       <c r="K15" s="6">
         <v>1</v>
@@ -1944,25 +1944,25 @@
         <v>178</v>
       </c>
       <c r="D21" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="H21" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="I21" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="J21" s="6" t="s">
         <v>184</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>185</v>
       </c>
       <c r="K21" s="6">
         <v>1</v>
@@ -2016,31 +2016,31 @@
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="H23" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="I23" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="J23" s="6" t="s">
         <v>192</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="J23" s="6" t="s">
-        <v>194</v>
       </c>
       <c r="K23" s="6">
         <v>1</v>
@@ -2094,31 +2094,31 @@
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>197</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>199</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>16</v>
       </c>
       <c r="H25" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="J25" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="K25" s="6">
         <v>1</v>
@@ -2178,23 +2178,23 @@
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="E27" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>206</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="K27" s="6">
         <v>1</v>
@@ -2254,31 +2254,31 @@
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="G29" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="H29" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="I29" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="J29" s="6" t="s">
         <v>214</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>216</v>
       </c>
       <c r="K29" s="6">
         <v>1</v>
@@ -2336,27 +2336,27 @@
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="E31" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="G31" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>222</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
       <c r="J31" s="6" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K31" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Release 1.0.3: rotación circular 4 eventos y clave coop online
- jugarPartida + multijugadorEventosCoop: ventana circular siempre 4 eventos.

- partidaCoop + multijugadorEventosCoop: event-rotation-coop-online-v1 para no cruzar completados con VS BOT.

- Versión 1.0.3, CHANGELOG; actualiza eventos.xlsx y eventos_online.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/eventos.xlsx
+++ b/public/resources/eventos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CEA91B-2D3D-492F-95EA-EEFD6EA73E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC7F659-A1FC-41A0-9EA2-679C73C4B2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="239">
   <si>
     <t>nombre</t>
   </si>
@@ -739,6 +739,9 @@
   </si>
   <si>
     <t>Psycho-Pirate</t>
+  </si>
+  <si>
+    <t>Hal Jordan</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1231,7 @@
         <v>30</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>31</v>
+        <v>238</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>32</v>

</xml_diff>